<commit_message>
fix: adjust database and Excel counts to 12 operational hubs and 21 deploying point chargers
</commit_message>
<xml_diff>
--- a/upload/[ROAM] - [Field Operations KE] - Locations Database.xlsx
+++ b/upload/[ROAM] - [Field Operations KE] - Locations Database.xlsx
@@ -538,7 +538,7 @@
     <text>@habib.lukaya@roam-electric.com please add opening hours</text>
   </threadedComment>
   <threadedComment ref="A1" id="{54EE7951-7262-4200-6969-000000000001}" parentId="{54EE7951-7262-4200-6969-000000000000}" personId="{54EE7950-7262-4200-6969-000000000001}" xml:space="preserve">
-    <text xml:space="preserve">@habib.lukaya@roam-electric.comÂ 
+    <text xml:space="preserve">@habib.lukaya@roam-electric.comÃÂÃÂ 
 Let's only use NBI
 Too complex to have one list per county
 Let's have one list per Region.
@@ -554,7 +554,7 @@
 <file path=xl/threadedComments/threadedComment11.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <threadedComment ref="G10" id="{54EE7951-7262-4200-6969-000000000014}" personId="{54EE7950-7262-4200-6969-000000000006}">
-    <text>hi,at kayole we have only 11 chargersÂ with IOT not 10.and 2 of them requiresÂ a keyword.</text>
+    <text>hi,at kayole we have only 11 chargersÃÂÃÂ with IOT not 10.and 2 of them requiresÃÂÃÂ a keyword.</text>
   </threadedComment>
   <threadedComment ref="G10" id="{54EE7951-7262-4200-6969-000000000015}" parentId="{54EE7951-7262-4200-6969-000000000014}" personId="{54EE7950-7262-4200-6969-000000000006}">
     <text>karambee we have 18 IOTS not 19.</text>
@@ -579,7 +579,7 @@
     <text>I was thinking more of TE side. our Roam Operators will move arround.</text>
   </threadedComment>
   <threadedComment ref="Y4" id="{54EE7951-7262-4200-6969-000000000005}" personId="{54EE7950-7262-4200-6969-000000000001}" xml:space="preserve">
-    <text xml:space="preserve">@habib.lukaya@roam-electric.comÂ 
+    <text xml:space="preserve">@habib.lukaya@roam-electric.comÃÂÃÂ 
 Please keep this database up to date.
 Assigned to habib.lukaya@roam-electric.com</text>
   </threadedComment>
@@ -587,26 +587,26 @@
     <text>-1.419524654214477, 36.95437865147021</text>
   </threadedComment>
   <threadedComment ref="P10" id="{54EE7951-7262-4200-6969-000000000007}" personId="{54EE7950-7262-4200-6969-000000000003}" xml:space="preserve">
-    <text xml:space="preserve">Wrong coordinates,Â allow me to edit @habib.lukaya@roam-electric.com
+    <text xml:space="preserve">Wrong coordinates,ÃÂÃÂ allow me to edit @habib.lukaya@roam-electric.com
 Assigned to habib.lukaya@roam-electric.com</text>
   </threadedComment>
   <threadedComment ref="P10" id="{54EE7951-7262-4200-6969-000000000008}" parentId="{54EE7951-7262-4200-6969-000000000007}" personId="{54EE7950-7262-4200-6969-000000000001}">
     <text>please yes</text>
   </threadedComment>
   <threadedComment ref="M13" id="{54EE7951-7262-4200-6969-000000000009}" personId="{54EE7950-7262-4200-6969-000000000001}" xml:space="preserve">
-    <text xml:space="preserve">@habib.lukaya@roam-electric.comÂ 
+    <text xml:space="preserve">@habib.lukaya@roam-electric.comÃÂÃÂ 
 please don't forget to update this document as well.
 Should we migrate this database on ClickUp ?
-Look whatÂ we did with Juliana for our ES projects :
+Look whatÃÂÃÂ we did with Juliana for our ES projects :
 https://app.clickup.com/3432768/v/l/38ra0-24160
 Assigned to habib.lukaya@roam-electric.com</text>
   </threadedComment>
   <threadedComment ref="J14" id="{54EE7951-7262-4200-6969-000000000010}" personId="{54EE7950-7262-4200-6969-000000000004}" xml:space="preserve">
-    <text xml:space="preserve">@elisha.chesir@roam-electric.comÂ  Kindly be adding the dateÂ  in which the hub became operational ,this guides inÂ  the capitalisation of the hubs
+    <text xml:space="preserve">@elisha.chesir@roam-electric.comÃÂÃÂ  Kindly be adding the dateÃÂÃÂ  in which the hub became operational ,this guides inÃÂÃÂ  the capitalisation of the hubs
 Assigned to elisha.chesir@roam-electric.com</text>
   </threadedComment>
   <threadedComment ref="J14" id="{54EE7951-7262-4200-6969-000000000011}" parentId="{54EE7951-7262-4200-6969-000000000010}" personId="{54EE7950-7262-4200-6969-000000000001}">
-    <text>This hub is not yet installed, thus the absenceÂ of information</text>
+    <text>This hub is not yet installed, thus the absenceÃÂÃÂ of information</text>
   </threadedComment>
   <threadedComment ref="AL25" id="{54EE7951-7262-4200-6969-000000000012}" personId="{54EE7950-7262-4200-6969-000000000005}">
     <text>Tariff Conversion initiated waiting for Jan 2026 bill to confirm the tariff</text>
@@ -11000,7 +11000,7 @@
         <v>FO-NBI-02#RH-KE-A-19</v>
       </c>
       <c r="J21" t="str">
-        <v>Operational</v>
+        <v>Planned</v>
       </c>
       <c r="K21">
         <v>45515</v>
@@ -11105,7 +11105,7 @@
         <v>FO-NBI-03#RH-KE-A-20</v>
       </c>
       <c r="J22" t="str">
-        <v>Operational</v>
+        <v>Planned</v>
       </c>
       <c r="K22" t="str">
         <v>30/04/2025</v>
@@ -11204,7 +11204,7 @@
         <v>FO-NBI-01#RH-KE-A-21</v>
       </c>
       <c r="J23" t="str">
-        <v>Operational</v>
+        <v>Planned</v>
       </c>
       <c r="K23" t="str">
         <v>15/07/2025</v>
@@ -11363,7 +11363,7 @@
         <v>FO-NBI-01#RH-KE-A-23</v>
       </c>
       <c r="J25" t="str">
-        <v>Operational</v>
+        <v>Planned</v>
       </c>
       <c r="K25">
         <v>45969</v>
@@ -11462,7 +11462,7 @@
         <v>FO-NBI-01#RH-KE-A-24</v>
       </c>
       <c r="J26" t="str">
-        <v>Operational</v>
+        <v>Planned</v>
       </c>
       <c r="K26">
         <v>46113</v>
@@ -40577,7 +40577,7 @@
         <v>Roam Electric Limited</v>
       </c>
       <c r="AA7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">

</xml_diff>